<commit_message>
Ajustes em backtests. em cofigs, algumas runs
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/backtest_results.xlsx
+++ b/pib_nowcast/data/backtest_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,179 +455,376 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>45992</v>
+        <v>45901</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45961</v>
+        <v>45869</v>
       </c>
       <c r="D2" t="n">
-        <v>1.59036854754432</v>
-      </c>
-      <c r="E2" t="n">
-        <v>192.94</v>
+        <v>1.671310055083186</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>pib    1.824705
+Name: 2025-09-01 00:00:00, dtype: float64</t>
+        </is>
       </c>
       <c r="F2" t="n">
-        <v>-23107.40604216351</v>
+        <v>-19234.12291496103</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>45992</v>
+        <v>45901</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>45991</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+        <v>45900</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.755624773923645</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>pib    1.824705
+Name: 2025-09-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>-19318.46773653902</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>45992</v>
+        <v>45901</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46022</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+        <v>45930</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.755697907491647</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>pib    1.824705
+Name: 2025-09-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>-19391.54996562334</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>45992</v>
+        <v>45901</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46053</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+        <v>45961</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.759777878485928</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>pib    1.824705
+Name: 2025-09-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>-19452.68360758301</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>45992</v>
+        <v>45901</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46081</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+        <v>45991</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.761310922581453</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>pib    1.824705
+Name: 2025-09-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>-19521.1895006021</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q4</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46082</v>
+        <v>45992</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46053</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+        <v>45961</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.42746407510225</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>pib    1.842175
+Name: 2025-12-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>-19452.68360758301</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q4</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46082</v>
+        <v>45992</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46081</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+        <v>45991</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.569333998716697</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>pib    1.842175
+Name: 2025-12-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>-19521.1895006021</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q4</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46082</v>
+        <v>45992</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46112</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+        <v>46022</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.568734038668366</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>pib    1.842175
+Name: 2025-12-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>-19578.02784234811</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q4</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46082</v>
+        <v>45992</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46142</v>
+        <v>46053</v>
       </c>
       <c r="D10" t="n">
-        <v>2.266792175434023</v>
-      </c>
-      <c r="E10" t="n">
-        <v>194.53</v>
+        <v>1.569477417657437</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>pib    1.842175
+Name: 2025-12-01 00:00:00, dtype: float64</t>
+        </is>
       </c>
       <c r="F10" t="n">
-        <v>-23718.94443309534</v>
+        <v>-19670.66746108279</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>2025Q4</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>46081</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.56949434873405</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>pib    1.842175
+Name: 2025-12-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>-19754.63566650098</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>2026Q1</t>
         </is>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B12" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C12" s="1" t="n">
+        <v>46053</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.807199580089058</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>pib    1.837504
+Name: 2026-03-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>-19670.66746108279</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>46081</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.848990565260393</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>pib    1.837504
+Name: 2026-03-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>-19754.63566650098</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>46112</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.843885606146172</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>pib    1.837504
+Name: 2026-03-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>-19863.54427225505</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.841050197074221</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>pib    1.837504
+Name: 2026-03-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>-19939.33238727939</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C16" s="1" t="n">
         <v>46173</v>
       </c>
-      <c r="D11" t="n">
-        <v>2.26385761156686</v>
-      </c>
-      <c r="E11" t="n">
-        <v>194.53</v>
-      </c>
-      <c r="F11" t="n">
-        <v>-23811.09615103708</v>
+      <c r="D16" t="n">
+        <v>1.840285643699618</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>pib    1.837504
+Name: 2026-03-01 00:00:00, dtype: float64</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>-20015.04623371518</v>
       </c>
     </row>
   </sheetData>

</xml_diff>